<commit_message>
feat: complete battleship ship and UI updates
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -3,13 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\放置\space-battleship\config_excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380"/>
+    <workbookView windowWidth="27945" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="config" sheetId="6" r:id="rId1"/>
@@ -32,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>name</t>
   </si>
@@ -88,25 +83,40 @@
     <t>死亡时后退距离</t>
   </si>
   <si>
+    <t>offlineMax</t>
+  </si>
+  <si>
+    <t>离线时长(h）</t>
+  </si>
+  <si>
+    <t>autoGenRes</t>
+  </si>
+  <si>
+    <t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</t>
+  </si>
+  <si>
+    <t>30,2,5,40</t>
+  </si>
+  <si>
+    <t>scientistCost</t>
+  </si>
+  <si>
+    <t>格式资源倍率,资源种类1|资源消耗1,资源种类2|资源消耗2....支持资源种类无限扩展</t>
+  </si>
+  <si>
+    <t>1.3,1|100,2|10</t>
+  </si>
+  <si>
     <t>hightechLimit</t>
   </si>
   <si>
-    <t>同时研发的高科技数量</t>
-  </si>
-  <si>
-    <t>offlineMax</t>
-  </si>
-  <si>
-    <t>离线时长(h）</t>
-  </si>
-  <si>
-    <t>autoGenRes</t>
-  </si>
-  <si>
-    <t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</t>
-  </si>
-  <si>
-    <t>30,2,5,40</t>
+    <t>高科技投入科学家的科研点数衰减</t>
+  </si>
+  <si>
+    <t>techPointGet</t>
+  </si>
+  <si>
+    <t>高科技点数获取</t>
   </si>
 </sst>
 </file>
@@ -1037,10 +1047,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.89166666666667" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="13.3796296296296" customWidth="1"/>
+    <col min="1" max="1" width="13.3833333333333" customWidth="1"/>
+    <col min="13" max="14" width="12.625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1139,7 +1150,7 @@
         <v>19</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1149,19 +1160,41 @@
       <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="C10">
-        <v>4</v>
+      <c r="C10" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sync local project and ignore generated files
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -1510,6 +1510,21 @@
         <v>1</v>
       </c>
     </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>hightechCostGrowthLevel</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>高科技耗时指数增长阈值，当前等级超过此值后生效</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>400</v>
+      </c>
+    </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Import explicit formation firing-space gap from official configuration workbook
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -1003,657 +1003,672 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C46"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.888889312744141" defaultRowHeight="14.39999961853027"/>
-  <cols>
-    <col width="48" customWidth="1" style="1" min="1" max="1"/>
-    <col width="42" customWidth="1" style="1" min="2" max="2"/>
-    <col width="49" customWidth="1" style="1" min="3" max="3"/>
-    <col width="12.62963008880615" customWidth="1" style="1" min="13" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" s="0" t="inlineStr">
-        <is>
-          <t>des</t>
-        </is>
-      </c>
-      <c r="C1" s="0" t="inlineStr">
-        <is>
-          <t>para_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t>这个配置的名字</t>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t>配置的描述</t>
-        </is>
-      </c>
-      <c r="C2" s="0" t="inlineStr">
-        <is>
-          <t>配置的参数</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t>如上</t>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>如上</t>
-        </is>
-      </c>
-      <c r="C3" s="0" t="inlineStr">
-        <is>
-          <t>如上</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="0" t="inlineStr">
-        <is>
-          <t>startEquip</t>
-        </is>
-      </c>
-      <c r="B4" s="0" t="inlineStr">
-        <is>
-          <t>飞船初始具有的装备，格式为name,name，equipment表的名字。默认为1级。</t>
-        </is>
-      </c>
-      <c r="C4" s="0" t="inlineStr">
-        <is>
-          <t>armour,laser</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="0" t="inlineStr">
-        <is>
-          <t>dmgReduce</t>
-        </is>
-      </c>
-      <c r="B5" s="0" t="inlineStr">
-        <is>
-          <t>护甲类型对应时，减少的伤害</t>
-        </is>
-      </c>
-      <c r="C5" s="0" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="0" t="inlineStr">
-        <is>
-          <t>movement</t>
-        </is>
-      </c>
-      <c r="B6" s="0" t="inlineStr">
-        <is>
-          <t>飞船的移动速度，单位是秒</t>
-        </is>
-      </c>
-      <c r="C6" s="0" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t>autoCollectReduce</t>
-        </is>
-      </c>
-      <c r="B7" s="0" t="inlineStr">
-        <is>
-          <t>自动拾取时的损耗</t>
-        </is>
-      </c>
-      <c r="C7" s="0" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="0" t="inlineStr">
-        <is>
-          <t>backRange</t>
-        </is>
-      </c>
-      <c r="B8" s="0" t="inlineStr">
-        <is>
-          <t>死亡时后退距离</t>
-        </is>
-      </c>
-      <c r="C8" s="0" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="0" t="inlineStr">
-        <is>
-          <t>offlineMax</t>
-        </is>
-      </c>
-      <c r="B9" s="0" t="inlineStr">
-        <is>
-          <t>离线时长(h）</t>
-        </is>
-      </c>
-      <c r="C9" s="0" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="0" t="inlineStr">
-        <is>
-          <t>autoGenRes</t>
-        </is>
-      </c>
-      <c r="B10" s="0" t="inlineStr">
-        <is>
-          <t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</t>
-        </is>
-      </c>
-      <c r="C10" s="0" t="inlineStr">
-        <is>
-          <t>30,2,5,40</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t>scientistCost</t>
-        </is>
-      </c>
-      <c r="B11" s="0" t="inlineStr">
-        <is>
-          <t>格式资源倍率,资源种类1|资源消耗1,资源种类2|资源消耗2....支持资源种类无限扩展</t>
-        </is>
-      </c>
-      <c r="C11" s="0" t="inlineStr">
-        <is>
-          <t>1.2,1|100,2|5</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="0" t="inlineStr">
-        <is>
-          <t>hightechLimit</t>
-        </is>
-      </c>
-      <c r="B12" s="0" t="inlineStr">
-        <is>
-          <t>高科技投入AI的科研点数衰减</t>
-        </is>
-      </c>
-      <c r="C12" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="0" t="inlineStr">
-        <is>
-          <t>techPointGet</t>
-        </is>
-      </c>
-      <c r="B13" s="0" t="inlineStr">
-        <is>
-          <t>高科技点数获取</t>
-        </is>
-      </c>
-      <c r="C13" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="0" t="inlineStr">
-        <is>
-          <t>hightechCostGrowthLevel</t>
-        </is>
-      </c>
-      <c r="B14" s="0" t="inlineStr">
-        <is>
-          <t>高科技耗时指数增长阈值，当前等级超过此值后生效</t>
-        </is>
-      </c>
-      <c r="C14" s="0" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="0" t="inlineStr">
-        <is>
-          <t>jewelDrop</t>
-        </is>
-      </c>
-      <c r="B15" s="0" t="inlineStr">
-        <is>
-          <t>宝石碎片掉率</t>
-        </is>
-      </c>
-      <c r="C15" s="0" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="inlineStr">
-        <is>
-          <t>chronoParticlesPerSecond</t>
-        </is>
-      </c>
-      <c r="B16" s="0" t="inlineStr">
-        <is>
-          <t>每离线秒获得的超时空微粒</t>
-        </is>
-      </c>
-      <c r="C16" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="0" t="inlineStr">
-        <is>
-          <t>chronoDefaultSpeed</t>
-        </is>
-      </c>
-      <c r="B17" s="0" t="inlineStr">
-        <is>
-          <t>进入游戏及微粒不足时恢复的倍率</t>
-        </is>
-      </c>
-      <c r="C17" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="0" t="inlineStr">
-        <is>
-          <t>chronoSpeeds</t>
-        </is>
-      </c>
-      <c r="B18" s="0" t="inlineStr">
-        <is>
-          <t>倍率|每现实秒微粒消耗，逗号分隔</t>
-        </is>
-      </c>
-      <c r="C18" s="0" t="inlineStr">
-        <is>
-          <t>1|0,2|1,3|2,4|3,5|4,6|5,7|6,8|7,9|8,10|9</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="0" t="inlineStr">
-        <is>
-          <t>reactorEnergyBase</t>
-        </is>
-      </c>
-      <c r="B19" s="0" t="inlineStr">
-        <is>
-          <t>反应炉1级总能源</t>
-        </is>
-      </c>
-      <c r="C19" s="0" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="inlineStr">
-        <is>
-          <t>reactorEnergyGrowth</t>
-        </is>
-      </c>
-      <c r="B20" s="0" t="inlineStr">
-        <is>
-          <t>反应炉每级总能源倍率</t>
-        </is>
-      </c>
-      <c r="C20" s="0" t="n">
-        <v>1.06</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t>reactorUpgradeBase</t>
-        </is>
-      </c>
-      <c r="B21" s="0" t="inlineStr">
-        <is>
-          <t>反应炉1级升级铀消耗</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="0" t="inlineStr">
-        <is>
-          <t>reactorUpgradeGrowth</t>
-        </is>
-      </c>
-      <c r="B22" s="0" t="inlineStr">
-        <is>
-          <t>反应炉每级升级费用倍率</t>
-        </is>
-      </c>
-      <c r="C22" s="0" t="n">
-        <v>1.35</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="0" t="inlineStr">
-        <is>
-          <t>reactorBoostExponent</t>
-        </is>
-      </c>
-      <c r="B23" s="0" t="inlineStr">
-        <is>
-          <t>模块能源提升指数；提升百分比为分配能源的该次幂</t>
-        </is>
-      </c>
-      <c r="C23" s="0" t="n">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="0" t="inlineStr">
-        <is>
-          <t>reactorUraniumId</t>
-        </is>
-      </c>
-      <c r="B24" s="0" t="inlineStr">
-        <is>
-          <t>反应炉升级消耗的资源ID</t>
-        </is>
-      </c>
-      <c r="C24" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="0" t="inlineStr">
-        <is>
-          <t>reactorModules</t>
-        </is>
-      </c>
-      <c r="B25" s="0" t="inlineStr">
-        <is>
-          <t>反应炉可分配模块ID，逗号分隔</t>
-        </is>
-      </c>
-      <c r="C25" s="0" t="inlineStr">
-        <is>
-          <t>weapons,defence,smelting,condensation</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="0" t="inlineStr">
-        <is>
-          <t>reactorInitialLevel</t>
-        </is>
-      </c>
-      <c r="B26" s="0" t="inlineStr">
-        <is>
-          <t>新存档反应炉初始等级</t>
-        </is>
-      </c>
-      <c r="C26" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="0" t="inlineStr">
-        <is>
-          <t>reactorPercentScale</t>
-        </is>
-      </c>
-      <c r="B27" s="0" t="inlineStr">
-        <is>
-          <t>提升百分比换算分母</t>
-        </is>
-      </c>
-      <c r="C27" s="0" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="0" t="inlineStr">
-        <is>
-          <t>reactorAllocationStep</t>
-        </is>
-      </c>
-      <c r="B28" s="0" t="inlineStr">
-        <is>
-          <t>能源滑杆最小步长</t>
-        </is>
-      </c>
-      <c r="C28" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="0" t="n"/>
-      <c r="B29" s="0" t="n"/>
-      <c r="C29" s="0" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="0" t="n"/>
-      <c r="B30" s="0" t="n"/>
-      <c r="C30" s="0" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="0" t="inlineStr">
-        <is>
-          <t>playerVisualScaleFrigate</t>
-        </is>
-      </c>
-      <c r="B31" s="0" t="inlineStr">
-        <is>
-          <t>我方护卫舰显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C31" s="0" t="n">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="0" t="inlineStr">
-        <is>
-          <t>playerVisualScaleDestroyer</t>
-        </is>
-      </c>
-      <c r="B32" s="0" t="inlineStr">
-        <is>
-          <t>我方驱逐舰显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C32" s="0" t="n">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="0" t="inlineStr">
-        <is>
-          <t>playerVisualScaleCruiser</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>我方巡洋舰显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C33" s="0" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1" s="1">
-      <c r="A34" s="0" t="inlineStr">
-        <is>
-          <t>playerVisualScaleBattleship</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>我方战列舰显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C34" s="0" t="n">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1" s="1">
-      <c r="A35" s="0" t="inlineStr">
-        <is>
-          <t>playerVisualScaleHeavy_Battleship</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>我方重型战列舰显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C35" s="0" t="n">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1" s="1">
-      <c r="A36" s="0" t="inlineStr">
-        <is>
-          <t>enemyVisualScaleSize1</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>敌方 size 1 显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C36" s="0" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1" s="1">
-      <c r="A37" s="0" t="inlineStr">
-        <is>
-          <t>enemyVisualScaleSize2</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>敌方 size 2 显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C37" s="0" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1" s="1">
-      <c r="A38" s="0" t="inlineStr">
-        <is>
-          <t>enemyVisualScaleSize3</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>敌方 size 3 显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C38" s="0" t="n">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1" s="1">
-      <c r="A39" s="0" t="inlineStr">
-        <is>
-          <t>enemyVisualScaleSize4</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>敌方 size 4 显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C39" s="0" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1" s="1">
-      <c r="A40" s="0" t="inlineStr">
-        <is>
-          <t>enemyVisualScaleSize5</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>敌方 size 5 显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C40" s="0" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1" s="1">
-      <c r="A41" s="0" t="inlineStr">
-        <is>
-          <t>enemyVisualScaleSize6</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>敌方 size 6 显示倍率，仅影响舰体贴图</t>
-        </is>
-      </c>
-      <c r="C41" s="0" t="n">
-        <v>1.7</v>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1" s="1">
-      <c r="A42" s="0" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="0" t="n"/>
-    </row>
-    <row r="43" ht="30" customHeight="1" s="1">
-      <c r="A43" s="0" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="0" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1" s="1">
-      <c r="A44" s="0" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="0" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1" s="1">
-      <c r="A45" s="0" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="0" t="n"/>
-    </row>
-    <row r="46" ht="30" customHeight="1" s="1">
-      <c r="A46" s="0" t="n"/>
-      <c r="B46" s="0" t="n"/>
-      <c r="C46" s="0" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
+    <ns0:pageSetUpPr/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:C47"/>
+  <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="8.888889312744141" defaultRowHeight="14.39999961853027"/>
+  <ns0:cols>
+    <ns0:col width="48" customWidth="1" style="1" min="1" max="1"/>
+    <ns0:col width="42" customWidth="1" style="1" min="2" max="2"/>
+    <ns0:col width="49" customWidth="1" style="1" min="3" max="3"/>
+    <ns0:col width="12.62963008880615" customWidth="1" style="1" min="13" max="14"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>name</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>des</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>para_1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>这个配置的名字</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>配置的描述</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>配置的参数</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>如上</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>如上</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>如上</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>startEquip</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>飞船初始具有的装备，格式为name,name，equipment表的名字。默认为1级。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>armour,laser</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>dmgReduce</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>护甲类型对应时，减少的伤害</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" s="0" t="n">
+        <ns0:v>0.5</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>movement</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>飞船的移动速度，单位是秒</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" s="0" t="n">
+        <ns0:v>50</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>autoCollectReduce</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>自动拾取时的损耗</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" s="0" t="n">
+        <ns0:v>0.5</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>backRange</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>死亡时后退距离</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" s="0" t="n">
+        <ns0:v>200</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>offlineMax</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>离线时长(h）</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" s="0" t="n">
+        <ns0:v>12</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>autoGenRes</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>30,2,5,40</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>scientistCost</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>格式资源倍率,资源种类1|资源消耗1,资源种类2|资源消耗2....支持资源种类无限扩展</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>1.2,1|100,2|5</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>hightechLimit</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>高科技投入AI的科研点数衰减</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" s="0" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>techPointGet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>高科技点数获取</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" s="0" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="A14" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>hightechCostGrowthLevel</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>高科技耗时指数增长阈值，当前等级超过此值后生效</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C14" s="0" t="n">
+        <ns0:v>50</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15">
+      <ns0:c r="A15" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jewelDrop</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>宝石碎片掉率</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C15" s="0" t="n">
+        <ns0:v>0.2</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16">
+      <ns0:c r="A16" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>chronoParticlesPerSecond</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>每离线秒获得的超时空微粒</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C16" s="0" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="A17" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>chronoDefaultSpeed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>进入游戏及微粒不足时恢复的倍率</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" s="0" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18">
+      <ns0:c r="A18" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>chronoSpeeds</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B18" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>倍率|每现实秒微粒消耗，逗号分隔</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C18" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>1|0,2|1,3|2,4|3,5|4,6|5,7|6,8|7,9|8,10|9</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19">
+      <ns0:c r="A19" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorEnergyBase</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B19" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>反应炉1级总能源</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C19" s="0" t="n">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20">
+      <ns0:c r="A20" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorEnergyGrowth</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B20" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>反应炉每级总能源倍率</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C20" s="0" t="n">
+        <ns0:v>1.06</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21">
+      <ns0:c r="A21" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorUpgradeBase</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B21" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>反应炉1级升级铀消耗</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C21" s="0" t="n">
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22">
+      <ns0:c r="A22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorUpgradeGrowth</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>反应炉每级升级费用倍率</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C22" s="0" t="n">
+        <ns0:v>1.35</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23">
+      <ns0:c r="A23" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorBoostExponent</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B23" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>模块能源提升指数；提升百分比为分配能源的该次幂</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C23" s="0" t="n">
+        <ns0:v>0.8</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24">
+      <ns0:c r="A24" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorUraniumId</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B24" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>反应炉升级消耗的资源ID</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C24" s="0" t="n">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25">
+      <ns0:c r="A25" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorModules</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B25" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>反应炉可分配模块ID，逗号分隔</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C25" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>weapons,defence,smelting,condensation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26">
+      <ns0:c r="A26" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorInitialLevel</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B26" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>新存档反应炉初始等级</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C26" s="0" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27">
+      <ns0:c r="A27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorPercentScale</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>提升百分比换算分母</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C27" s="0" t="n">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reactorAllocationStep</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>能源滑杆最小步长</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C28" s="0" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29">
+      <ns0:c r="A29" s="0" t="n"/>
+      <ns0:c r="B29" s="0" t="n"/>
+      <ns0:c r="C29" s="0" t="n"/>
+    </ns0:row>
+    <ns0:row r="30">
+      <ns0:c r="A30" s="0" t="n"/>
+      <ns0:c r="B30" s="0" t="n"/>
+      <ns0:c r="C30" s="0" t="n"/>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>playerVisualScaleFrigate</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>我方护卫舰显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C31" s="0" t="n">
+        <ns0:v>1.3</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32">
+      <ns0:c r="A32" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>playerVisualScaleDestroyer</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B32" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>我方驱逐舰显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C32" s="0" t="n">
+        <ns0:v>1.1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33">
+      <ns0:c r="A33" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>playerVisualScaleCruiser</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B33" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>我方巡洋舰显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C33" s="0" t="n">
+        <ns0:v>1.2</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34" ht="30" customHeight="1" s="1">
+      <ns0:c r="A34" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>playerVisualScaleBattleship</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B34" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>我方战列舰显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C34" s="0" t="n">
+        <ns0:v>1.3</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="35" ht="30" customHeight="1" s="1">
+      <ns0:c r="A35" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>playerVisualScaleHeavy_Battleship</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B35" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>我方重型战列舰显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C35" s="0" t="n">
+        <ns0:v>1.4</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="36" ht="30" customHeight="1" s="1">
+      <ns0:c r="A36" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>enemyVisualScaleSize1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B36" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>敌方 size 1 显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C36" s="0" t="n">
+        <ns0:v>1.2</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="37" ht="30" customHeight="1" s="1">
+      <ns0:c r="A37" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>enemyVisualScaleSize2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B37" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>敌方 size 2 显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C37" s="0" t="n">
+        <ns0:v>1.2</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="38" ht="30" customHeight="1" s="1">
+      <ns0:c r="A38" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>enemyVisualScaleSize3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B38" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>敌方 size 3 显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C38" s="0" t="n">
+        <ns0:v>1.4</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="39" ht="30" customHeight="1" s="1">
+      <ns0:c r="A39" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>enemyVisualScaleSize4</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B39" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>敌方 size 4 显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C39" s="0" t="n">
+        <ns0:v>1.5</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="40" ht="30" customHeight="1" s="1">
+      <ns0:c r="A40" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>enemyVisualScaleSize5</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B40" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>敌方 size 5 显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C40" s="0" t="n">
+        <ns0:v>1.5</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="41" ht="30" customHeight="1" s="1">
+      <ns0:c r="A41" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>enemyVisualScaleSize6</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B41" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>敌方 size 6 显示倍率，仅影响舰体贴图</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C41" s="0" t="n">
+        <ns0:v>1.7</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="42" ht="30" customHeight="1" s="1">
+      <ns0:c r="A42" s="0" t="n"/>
+      <ns0:c r="B42" s="2" t="n"/>
+      <ns0:c r="C42" s="0" t="n"/>
+    </ns0:row>
+    <ns0:row r="43" ht="30" customHeight="1" s="1">
+      <ns0:c r="A43" s="0" t="n"/>
+      <ns0:c r="B43" s="2" t="n"/>
+      <ns0:c r="C43" s="0" t="n"/>
+    </ns0:row>
+    <ns0:row r="44" ht="30" customHeight="1" s="1">
+      <ns0:c r="A44" s="0" t="n"/>
+      <ns0:c r="B44" s="2" t="n"/>
+      <ns0:c r="C44" s="0" t="n"/>
+    </ns0:row>
+    <ns0:row r="45" ht="30" customHeight="1" s="1">
+      <ns0:c r="A45" s="0" t="n"/>
+      <ns0:c r="B45" s="2" t="n"/>
+      <ns0:c r="C45" s="0" t="n"/>
+    </ns0:row>
+    <ns0:row r="46" ht="30" customHeight="1" s="1">
+      <ns0:c r="A46" s="0" t="n"/>
+      <ns0:c r="B46" s="0" t="n"/>
+      <ns0:c r="C46" s="0" t="n"/>
+    </ns0:row>
+    <ns0:row r="47">
+      <ns0:c r="A47" t="inlineStr">
+        <ns0:is>
+          <ns0:t>explicitEnemyPlayerMinGap</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B47" t="inlineStr">
+        <ns0:is>
+          <ns0:t>显式超空间阵型与玩家舰体包络的最小发射空白，按战场高度比例；不改变普通阵型、船体尺寸或战斗数值。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C47">
+        <ns0:v>0.12</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
Make early research and reactor growth tangible while preserving power shares
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -1003,672 +1003,672 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr/>
-  </ns0:sheetPr>
-  <ns0:dimension ref="A1:C47"/>
-  <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="8.888889312744141" defaultRowHeight="14.39999961853027"/>
-  <ns0:cols>
-    <ns0:col width="48" customWidth="1" style="1" min="1" max="1"/>
-    <ns0:col width="42" customWidth="1" style="1" min="2" max="2"/>
-    <ns0:col width="49" customWidth="1" style="1" min="3" max="3"/>
-    <ns0:col width="12.62963008880615" customWidth="1" style="1" min="13" max="14"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="A1" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B1" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>des</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C1" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>para_1</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2">
-      <ns0:c r="A2" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>这个配置的名字</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B2" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>配置的描述</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C2" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>配置的参数</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3">
-      <ns0:c r="A3" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>如上</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>如上</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C3" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>如上</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4">
-      <ns0:c r="A4" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>startEquip</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B4" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>飞船初始具有的装备，格式为name,name，equipment表的名字。默认为1级。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C4" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>armour,laser</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5">
-      <ns0:c r="A5" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dmgReduce</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>护甲类型对应时，减少的伤害</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C5" s="0" t="n">
-        <ns0:v>0.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="6">
-      <ns0:c r="A6" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>movement</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B6" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>飞船的移动速度，单位是秒</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C6" s="0" t="n">
-        <ns0:v>50</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>autoCollectReduce</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B7" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>自动拾取时的损耗</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C7" s="0" t="n">
-        <ns0:v>0.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8">
-      <ns0:c r="A8" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>backRange</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B8" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>死亡时后退距离</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C8" s="0" t="n">
-        <ns0:v>200</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="9">
-      <ns0:c r="A9" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>offlineMax</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B9" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>离线时长(h）</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C9" s="0" t="n">
-        <ns0:v>12</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10">
-      <ns0:c r="A10" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>autoGenRes</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B10" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C10" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>30,2,5,40</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11">
-      <ns0:c r="A11" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>scientistCost</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B11" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>格式资源倍率,资源种类1|资源消耗1,资源种类2|资源消耗2....支持资源种类无限扩展</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C11" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>1.2,1|100,2|5</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="12">
-      <ns0:c r="A12" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hightechLimit</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B12" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>高科技投入AI的科研点数衰减</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C12" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="13">
-      <ns0:c r="A13" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>techPointGet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B13" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>高科技点数获取</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C13" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="A14" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hightechCostGrowthLevel</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B14" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>高科技耗时指数增长阈值，当前等级超过此值后生效</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C14" s="0" t="n">
-        <ns0:v>50</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="15">
-      <ns0:c r="A15" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jewelDrop</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B15" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>宝石碎片掉率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C15" s="0" t="n">
-        <ns0:v>0.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16">
-      <ns0:c r="A16" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chronoParticlesPerSecond</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B16" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>每离线秒获得的超时空微粒</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C16" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="17">
-      <ns0:c r="A17" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chronoDefaultSpeed</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B17" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>进入游戏及微粒不足时恢复的倍率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C17" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="18">
-      <ns0:c r="A18" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chronoSpeeds</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B18" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>倍率|每现实秒微粒消耗，逗号分隔</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C18" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>1|0,2|1,3|2,4|3,5|4,6|5,7|6,8|7,9|8,10|9</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="19">
-      <ns0:c r="A19" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorEnergyBase</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B19" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉1级总能源</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C19" s="0" t="n">
-        <ns0:v>100</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="20">
-      <ns0:c r="A20" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorEnergyGrowth</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B20" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉每级总能源倍率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C20" s="0" t="n">
-        <ns0:v>1.06</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="21">
-      <ns0:c r="A21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorUpgradeBase</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉1级升级铀消耗</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C21" s="0" t="n">
-        <ns0:v>10</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="22">
-      <ns0:c r="A22" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorUpgradeGrowth</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B22" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉每级升级费用倍率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C22" s="0" t="n">
-        <ns0:v>1.35</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="23">
-      <ns0:c r="A23" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorBoostExponent</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B23" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>模块能源提升指数；提升百分比为分配能源的该次幂</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C23" s="0" t="n">
-        <ns0:v>0.8</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="24">
-      <ns0:c r="A24" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorUraniumId</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B24" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉升级消耗的资源ID</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C24" s="0" t="n">
-        <ns0:v>2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="25">
-      <ns0:c r="A25" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorModules</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B25" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉可分配模块ID，逗号分隔</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C25" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>weapons,defence,smelting,condensation</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="26">
-      <ns0:c r="A26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorInitialLevel</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>新存档反应炉初始等级</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C26" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="27">
-      <ns0:c r="A27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorPercentScale</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>提升百分比换算分母</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C27" s="0" t="n">
-        <ns0:v>100</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28">
-      <ns0:c r="A28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorAllocationStep</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>能源滑杆最小步长</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C28" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="29">
-      <ns0:c r="A29" s="0" t="n"/>
-      <ns0:c r="B29" s="0" t="n"/>
-      <ns0:c r="C29" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="30">
-      <ns0:c r="A30" s="0" t="n"/>
-      <ns0:c r="B30" s="0" t="n"/>
-      <ns0:c r="C30" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="31">
-      <ns0:c r="A31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleFrigate</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方护卫舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C31" s="0" t="n">
-        <ns0:v>1.3</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="32">
-      <ns0:c r="A32" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleDestroyer</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B32" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方驱逐舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C32" s="0" t="n">
-        <ns0:v>1.1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="33">
-      <ns0:c r="A33" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleCruiser</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B33" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方巡洋舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C33" s="0" t="n">
-        <ns0:v>1.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="34" ht="30" customHeight="1" s="1">
-      <ns0:c r="A34" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleBattleship</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B34" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方战列舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C34" s="0" t="n">
-        <ns0:v>1.3</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="35" ht="30" customHeight="1" s="1">
-      <ns0:c r="A35" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleHeavy_Battleship</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B35" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方重型战列舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C35" s="0" t="n">
-        <ns0:v>1.4</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="36" ht="30" customHeight="1" s="1">
-      <ns0:c r="A36" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize1</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B36" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 1 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C36" s="0" t="n">
-        <ns0:v>1.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="37" ht="30" customHeight="1" s="1">
-      <ns0:c r="A37" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize2</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B37" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 2 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C37" s="0" t="n">
-        <ns0:v>1.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="38" ht="30" customHeight="1" s="1">
-      <ns0:c r="A38" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize3</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B38" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 3 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C38" s="0" t="n">
-        <ns0:v>1.4</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="39" ht="30" customHeight="1" s="1">
-      <ns0:c r="A39" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize4</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B39" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 4 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C39" s="0" t="n">
-        <ns0:v>1.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="40" ht="30" customHeight="1" s="1">
-      <ns0:c r="A40" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize5</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B40" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 5 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C40" s="0" t="n">
-        <ns0:v>1.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="41" ht="30" customHeight="1" s="1">
-      <ns0:c r="A41" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize6</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B41" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 6 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C41" s="0" t="n">
-        <ns0:v>1.7</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="42" ht="30" customHeight="1" s="1">
-      <ns0:c r="A42" s="0" t="n"/>
-      <ns0:c r="B42" s="2" t="n"/>
-      <ns0:c r="C42" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="43" ht="30" customHeight="1" s="1">
-      <ns0:c r="A43" s="0" t="n"/>
-      <ns0:c r="B43" s="2" t="n"/>
-      <ns0:c r="C43" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="44" ht="30" customHeight="1" s="1">
-      <ns0:c r="A44" s="0" t="n"/>
-      <ns0:c r="B44" s="2" t="n"/>
-      <ns0:c r="C44" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="45" ht="30" customHeight="1" s="1">
-      <ns0:c r="A45" s="0" t="n"/>
-      <ns0:c r="B45" s="2" t="n"/>
-      <ns0:c r="C45" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="46" ht="30" customHeight="1" s="1">
-      <ns0:c r="A46" s="0" t="n"/>
-      <ns0:c r="B46" s="0" t="n"/>
-      <ns0:c r="C46" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="47">
-      <ns0:c r="A47" t="inlineStr">
-        <ns0:is>
-          <ns0:t>explicitEnemyPlayerMinGap</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B47" t="inlineStr">
-        <ns0:is>
-          <ns0:t>显式超空间阵型与玩家舰体包络的最小发射空白，按战场高度比例；不改变普通阵型、船体尺寸或战斗数值。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C47">
-        <ns0:v>0.12</ns0:v>
-      </ns0:c>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C47"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.888889312744141" defaultRowHeight="14.39999961853027"/>
+  <cols>
+    <col width="48" customWidth="1" style="1" min="1" max="1"/>
+    <col width="42" customWidth="1" style="1" min="2" max="2"/>
+    <col width="49" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12.62963008880615" customWidth="1" style="1" min="13" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>des</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>para_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>这个配置的名字</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>配置的描述</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>配置的参数</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>如上</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>如上</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>如上</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>startEquip</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>飞船初始具有的装备，格式为name,name，equipment表的名字。默认为1级。</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>armour,laser</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>dmgReduce</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>护甲类型对应时，减少的伤害</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>飞船的移动速度，单位是秒</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>autoCollectReduce</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>自动拾取时的损耗</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>backRange</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>死亡时后退距离</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>offlineMax</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>离线时长(h）</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>autoGenRes</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>30,2,5,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>scientistCost</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>格式资源倍率,资源种类1|资源消耗1,资源种类2|资源消耗2....支持资源种类无限扩展</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>1.2,1|100,2|5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>hightechLimit</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>高科技投入AI的科研点数衰减</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>techPointGet</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>高科技点数获取</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>hightechCostGrowthLevel</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>高科技耗时指数增长阈值，当前等级超过此值后生效</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>jewelDrop</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>宝石碎片掉率</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>chronoParticlesPerSecond</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>每离线秒获得的超时空微粒</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>chronoDefaultSpeed</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>进入游戏及微粒不足时恢复的倍率</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>chronoSpeeds</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>倍率|每现实秒微粒消耗，逗号分隔</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>1|0,2|1,3|2,4|3,5|4,6|5,7|6,8|7,9|8,10|9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>reactorEnergyBase</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>反应炉1级总能源</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>reactorEnergyGrowth</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>反应炉每级总能源倍率</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>reactorUpgradeBase</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>反应炉1级升级铀消耗</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>reactorUpgradeGrowth</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>反应炉每级升级费用倍率</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>reactorBoostExponent</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>模块能源提升指数；提升百分比为分配能源的该次幂</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>reactorUraniumId</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>反应炉升级消耗的资源ID</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>reactorModules</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>反应炉可分配模块ID，逗号分隔</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>weapons,defence,smelting,condensation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>reactorInitialLevel</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>新存档反应炉初始等级</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>reactorPercentScale</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>提升百分比换算分母</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>reactorAllocationStep</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>能源滑杆最小步长</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n"/>
+      <c r="B29" s="0" t="n"/>
+      <c r="C29" s="0" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n"/>
+      <c r="B30" s="0" t="n"/>
+      <c r="C30" s="0" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleFrigate</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>我方护卫舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleDestroyer</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>我方驱逐舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleCruiser</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>我方巡洋舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1" s="1">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleBattleship</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>我方战列舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1" s="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleHeavy_Battleship</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>我方重型战列舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1" s="1">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize1</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 1 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1" s="1">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize2</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 2 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1" s="1">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize3</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 3 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1" s="1">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize4</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 4 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1" s="1">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize5</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 5 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1" s="1">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize6</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 6 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1" s="1">
+      <c r="A42" s="0" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="0" t="n"/>
+    </row>
+    <row r="43" ht="30" customHeight="1" s="1">
+      <c r="A43" s="0" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="0" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1" s="1">
+      <c r="A44" s="0" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="0" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1" s="1">
+      <c r="A45" s="0" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="0" t="n"/>
+    </row>
+    <row r="46" ht="30" customHeight="1" s="1">
+      <c r="A46" s="0" t="n"/>
+      <c r="B46" s="0" t="n"/>
+      <c r="C46" s="0" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>explicitEnemyPlayerMinGap</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>显式超空间阵型与玩家舰体包络的最小发射空白，按战场高度比例；不改变普通阵型、船体尺寸或战斗数值。</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Integrate playability and promotion workflow candidates for continued QA
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -1003,672 +1003,672 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr/>
-  </ns0:sheetPr>
-  <ns0:dimension ref="A1:C47"/>
-  <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="8.888889312744141" defaultRowHeight="14.39999961853027"/>
-  <ns0:cols>
-    <ns0:col width="48" customWidth="1" style="1" min="1" max="1"/>
-    <ns0:col width="42" customWidth="1" style="1" min="2" max="2"/>
-    <ns0:col width="49" customWidth="1" style="1" min="3" max="3"/>
-    <ns0:col width="12.62963008880615" customWidth="1" style="1" min="13" max="14"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="A1" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B1" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>des</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C1" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>para_1</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2">
-      <ns0:c r="A2" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>这个配置的名字</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B2" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>配置的描述</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C2" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>配置的参数</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3">
-      <ns0:c r="A3" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>如上</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>如上</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C3" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>如上</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4">
-      <ns0:c r="A4" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>startEquip</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B4" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>飞船初始具有的装备，格式为name,name，equipment表的名字。默认为1级。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C4" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>armour,laser</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5">
-      <ns0:c r="A5" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dmgReduce</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>护甲类型对应时，减少的伤害</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C5" s="0" t="n">
-        <ns0:v>0.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="6">
-      <ns0:c r="A6" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>movement</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B6" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>飞船的移动速度，单位是秒</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C6" s="0" t="n">
-        <ns0:v>50</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>autoCollectReduce</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B7" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>自动拾取时的损耗</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C7" s="0" t="n">
-        <ns0:v>0.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8">
-      <ns0:c r="A8" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>backRange</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B8" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>死亡时后退距离</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C8" s="0" t="n">
-        <ns0:v>200</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="9">
-      <ns0:c r="A9" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>offlineMax</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B9" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>离线时长(h）</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C9" s="0" t="n">
-        <ns0:v>12</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10">
-      <ns0:c r="A10" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>autoGenRes</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B10" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C10" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>30,2,5,40</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11">
-      <ns0:c r="A11" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>scientistCost</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B11" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>格式资源倍率,资源种类1|资源消耗1,资源种类2|资源消耗2....支持资源种类无限扩展</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C11" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>1.2,1|100,2|5</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="12">
-      <ns0:c r="A12" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hightechLimit</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B12" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>高科技投入AI的科研点数衰减</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C12" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="13">
-      <ns0:c r="A13" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>techPointGet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B13" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>高科技点数获取</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C13" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="A14" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hightechCostGrowthLevel</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B14" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>高科技耗时指数增长阈值，当前等级超过此值后生效</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C14" s="0" t="n">
-        <ns0:v>50</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="15">
-      <ns0:c r="A15" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jewelDrop</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B15" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>宝石碎片掉率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C15" s="0" t="n">
-        <ns0:v>0.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16">
-      <ns0:c r="A16" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chronoParticlesPerSecond</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B16" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>每离线秒获得的超时空微粒</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C16" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="17">
-      <ns0:c r="A17" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chronoDefaultSpeed</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B17" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>进入游戏及微粒不足时恢复的倍率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C17" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="18">
-      <ns0:c r="A18" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chronoSpeeds</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B18" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>倍率|每现实秒微粒消耗，逗号分隔</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C18" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>1|0,2|1,3|2,4|3,5|4,6|5,7|6,8|7,9|8,10|9</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="19">
-      <ns0:c r="A19" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorEnergyBase</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B19" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉1级总能源</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C19" s="0" t="n">
-        <ns0:v>100</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="20">
-      <ns0:c r="A20" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorEnergyGrowth</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B20" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉每级总能源倍率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C20" s="0" t="n">
-        <ns0:v>1.06</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="21">
-      <ns0:c r="A21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorUpgradeBase</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉1级升级铀消耗</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C21" s="0" t="n">
-        <ns0:v>10</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="22">
-      <ns0:c r="A22" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorUpgradeGrowth</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B22" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉每级升级费用倍率</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C22" s="0" t="n">
-        <ns0:v>1.35</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="23">
-      <ns0:c r="A23" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorBoostExponent</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B23" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>模块能源提升指数；提升百分比为分配能源的该次幂</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C23" s="0" t="n">
-        <ns0:v>0.8</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="24">
-      <ns0:c r="A24" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorUraniumId</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B24" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉升级消耗的资源ID</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C24" s="0" t="n">
-        <ns0:v>2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="25">
-      <ns0:c r="A25" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorModules</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B25" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反应炉可分配模块ID，逗号分隔</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C25" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>weapons,defence,smelting,condensation</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="26">
-      <ns0:c r="A26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorInitialLevel</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>新存档反应炉初始等级</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C26" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="27">
-      <ns0:c r="A27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorPercentScale</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>提升百分比换算分母</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C27" s="0" t="n">
-        <ns0:v>100</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28">
-      <ns0:c r="A28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reactorAllocationStep</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>能源滑杆最小步长</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C28" s="0" t="n">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="29">
-      <ns0:c r="A29" s="0" t="n"/>
-      <ns0:c r="B29" s="0" t="n"/>
-      <ns0:c r="C29" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="30">
-      <ns0:c r="A30" s="0" t="n"/>
-      <ns0:c r="B30" s="0" t="n"/>
-      <ns0:c r="C30" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="31">
-      <ns0:c r="A31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleFrigate</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方护卫舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C31" s="0" t="n">
-        <ns0:v>1.3</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="32">
-      <ns0:c r="A32" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleDestroyer</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B32" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方驱逐舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C32" s="0" t="n">
-        <ns0:v>1.1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="33">
-      <ns0:c r="A33" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleCruiser</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B33" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方巡洋舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C33" s="0" t="n">
-        <ns0:v>1.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="34" ht="30" customHeight="1" s="1">
-      <ns0:c r="A34" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleBattleship</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B34" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方战列舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C34" s="0" t="n">
-        <ns0:v>1.3</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="35" ht="30" customHeight="1" s="1">
-      <ns0:c r="A35" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>playerVisualScaleHeavy_Battleship</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B35" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>我方重型战列舰显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C35" s="0" t="n">
-        <ns0:v>1.4</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="36" ht="30" customHeight="1" s="1">
-      <ns0:c r="A36" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize1</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B36" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 1 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C36" s="0" t="n">
-        <ns0:v>1.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="37" ht="30" customHeight="1" s="1">
-      <ns0:c r="A37" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize2</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B37" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 2 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C37" s="0" t="n">
-        <ns0:v>1.2</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="38" ht="30" customHeight="1" s="1">
-      <ns0:c r="A38" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize3</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B38" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 3 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C38" s="0" t="n">
-        <ns0:v>1.4</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="39" ht="30" customHeight="1" s="1">
-      <ns0:c r="A39" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize4</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B39" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 4 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C39" s="0" t="n">
-        <ns0:v>1.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="40" ht="30" customHeight="1" s="1">
-      <ns0:c r="A40" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize5</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B40" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 5 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C40" s="0" t="n">
-        <ns0:v>1.5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="41" ht="30" customHeight="1" s="1">
-      <ns0:c r="A41" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t>enemyVisualScaleSize6</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B41" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>敌方 size 6 显示倍率，仅影响舰体贴图</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C41" s="0" t="n">
-        <ns0:v>1.7</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="42" ht="30" customHeight="1" s="1">
-      <ns0:c r="A42" s="0" t="n"/>
-      <ns0:c r="B42" s="2" t="n"/>
-      <ns0:c r="C42" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="43" ht="30" customHeight="1" s="1">
-      <ns0:c r="A43" s="0" t="n"/>
-      <ns0:c r="B43" s="2" t="n"/>
-      <ns0:c r="C43" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="44" ht="30" customHeight="1" s="1">
-      <ns0:c r="A44" s="0" t="n"/>
-      <ns0:c r="B44" s="2" t="n"/>
-      <ns0:c r="C44" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="45" ht="30" customHeight="1" s="1">
-      <ns0:c r="A45" s="0" t="n"/>
-      <ns0:c r="B45" s="2" t="n"/>
-      <ns0:c r="C45" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="46" ht="30" customHeight="1" s="1">
-      <ns0:c r="A46" s="0" t="n"/>
-      <ns0:c r="B46" s="0" t="n"/>
-      <ns0:c r="C46" s="0" t="n"/>
-    </ns0:row>
-    <ns0:row r="47">
-      <ns0:c r="A47" t="inlineStr">
-        <ns0:is>
-          <ns0:t>explicitEnemyPlayerMinGap</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B47" t="inlineStr">
-        <ns0:is>
-          <ns0:t>显式超空间阵型与玩家舰体包络的最小发射空白，按战场高度比例；不改变普通阵型、船体尺寸或战斗数值。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C47">
-        <ns0:v>0.12</ns0:v>
-      </ns0:c>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C47"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.888889312744141" defaultRowHeight="14.39999961853027"/>
+  <cols>
+    <col width="48" customWidth="1" style="1" min="1" max="1"/>
+    <col width="42" customWidth="1" style="1" min="2" max="2"/>
+    <col width="49" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12.62963008880615" customWidth="1" style="1" min="13" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>des</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>para_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>这个配置的名字</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>配置的描述</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>配置的参数</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>如上</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>如上</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>如上</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>startEquip</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>飞船初始具有的装备，格式为name,name，equipment表的名字。默认为1级。</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>armour,laser</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>dmgReduce</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>护甲类型对应时，减少的伤害</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>飞船的移动速度，单位是秒</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>autoCollectReduce</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>自动拾取时的损耗</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>backRange</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>死亡时后退距离</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>offlineMax</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>离线时长(h）</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>autoGenRes</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>画面上自动生成的资源,格式为生成间隔秒,种类,数量,移动速度.</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>30,2,5,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>scientistCost</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>格式资源倍率,资源种类1|资源消耗1,资源种类2|资源消耗2....支持资源种类无限扩展</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>1.2,1|100,2|5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>hightechLimit</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>高科技投入AI的科研点数衰减</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>techPointGet</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>高科技点数获取</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>hightechCostGrowthLevel</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>高科技耗时指数增长阈值，当前等级超过此值后生效</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>jewelDrop</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>宝石碎片掉率</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>chronoParticlesPerSecond</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>每离线秒获得的超时空微粒</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>chronoDefaultSpeed</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>进入游戏及微粒不足时恢复的倍率</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>chronoSpeeds</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>倍率|每现实秒微粒消耗，逗号分隔</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>1|0,2|1,3|2,4|3,5|4,6|5,7|6,8|7,9|8,10|9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>reactorEnergyBase</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>反应炉1级总能源</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>reactorEnergyGrowth</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>反应炉每级总能源倍率</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>reactorUpgradeBase</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>反应炉1级升级铀消耗</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>reactorUpgradeGrowth</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>反应炉每级升级费用倍率</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>reactorBoostExponent</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>模块能源提升指数；提升百分比为分配能源的该次幂</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>reactorUraniumId</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>反应炉升级消耗的资源ID</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>reactorModules</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>反应炉可分配模块ID，逗号分隔</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>weapons,defence,smelting,condensation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>reactorInitialLevel</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>新存档反应炉初始等级</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>reactorPercentScale</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>提升百分比换算分母</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>reactorAllocationStep</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>能源滑杆最小步长</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n"/>
+      <c r="B29" s="0" t="n"/>
+      <c r="C29" s="0" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n"/>
+      <c r="B30" s="0" t="n"/>
+      <c r="C30" s="0" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleFrigate</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>我方护卫舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleDestroyer</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>我方驱逐舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleCruiser</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>我方巡洋舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1" s="1">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleBattleship</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>我方战列舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1" s="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>playerVisualScaleHeavy_Battleship</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>我方重型战列舰显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1" s="1">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize1</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 1 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1" s="1">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize2</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 2 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1" s="1">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize3</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 3 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1" s="1">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize4</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 4 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1" s="1">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize5</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 5 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1" s="1">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>enemyVisualScaleSize6</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>敌方 size 6 显示倍率，仅影响舰体贴图</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1" s="1">
+      <c r="A42" s="0" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="0" t="n"/>
+    </row>
+    <row r="43" ht="30" customHeight="1" s="1">
+      <c r="A43" s="0" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="0" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1" s="1">
+      <c r="A44" s="0" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="0" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1" s="1">
+      <c r="A45" s="0" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="0" t="n"/>
+    </row>
+    <row r="46" ht="30" customHeight="1" s="1">
+      <c r="A46" s="0" t="n"/>
+      <c r="B46" s="0" t="n"/>
+      <c r="C46" s="0" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>explicitEnemyPlayerMinGap</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>显式超空间阵型与玩家舰体包络的最小发射空白，按战场高度比例；不改变普通阵型、船体尺寸或战斗数值。</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Trial uniform reactor capacity growth at 1.20 with safe purchase bounds
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -1324,11 +1324,11 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>反应炉每级总能源倍率</t>
+          <t>反应炉每级总能源倍率；同等级按当前配置统一计算</t>
         </is>
       </c>
       <c r="C20" s="0" t="n">
-        <v>1.06</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Trial reactor growth and compact upgrade-return preview candidate
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -1324,11 +1324,11 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>反应炉每级总能源倍率</t>
+          <t>反应炉每级总能源倍率；同等级按当前配置统一计算</t>
         </is>
       </c>
       <c r="C20" s="0" t="n">
-        <v>1.06</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Restore original AI unlock gates and add per-slot refit cooldown
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/config.xlsx
+++ b/space-battleship/config_excel/config.xlsx
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.888889312744141" defaultRowHeight="14.39999961853027"/>
   <cols>
     <col width="48" customWidth="1" style="1" min="1" max="1"/>
@@ -1668,6 +1668,21 @@
         <v>0.12</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>equipmentSwitchCooldownSeconds</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>同一武器或防御槽位换装后再次换装的游戏秒数</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="n">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>